<commit_message>
Fixed Negatives in Order Profit Calculation
</commit_message>
<xml_diff>
--- a/faker/categories.xlsx
+++ b/faker/categories.xlsx
@@ -505,7 +505,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Wholesale</t>
+          <t>Limited Edition</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -553,7 +553,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Budget</t>
+          <t>On Discount</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -601,7 +601,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Limited Edition</t>
+          <t>Special Offer</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -649,7 +649,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Retail</t>
+          <t>Budget</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -697,7 +697,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Featured</t>
+          <t>New Arrival</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -747,7 +747,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Premium  </t>
+          <t xml:space="preserve">  Featured  </t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -797,7 +797,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>On Discount</t>
+          <t>Sale</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -847,7 +847,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Limited Edition</t>
+          <t>Special Offer</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -895,7 +895,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>New Arrival</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -945,7 +945,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Professional</t>
+          <t>Clearance</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -995,7 +995,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Clearance@</t>
+          <t>Regular@</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1045,7 +1045,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>New Arrival</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1093,7 +1093,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Professional</t>
+          <t>Clearance</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1141,7 +1141,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>Featured</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1189,7 +1189,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Consumer</t>
+          <t>Industrial</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1237,7 +1237,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Retail</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1285,7 +1285,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Sale</t>
+          <t>Wholesale</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1385,7 +1385,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>On Discount</t>
+          <t>Sale</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1433,7 +1433,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Regular</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1481,7 +1481,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Industrial  </t>
+          <t xml:space="preserve">  Retail  </t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1531,7 +1531,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Featured</t>
+          <t>New Arrival</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1579,7 +1579,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Special Offer</t>
+          <t>Professional</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1629,7 +1629,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Clearance</t>
+          <t>Regular</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1677,7 +1677,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Retail</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1727,7 +1727,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>CONSUMER</t>
+          <t>INDUSTRIAL</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1775,7 +1775,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Consumer  </t>
+          <t xml:space="preserve">  Industrial  </t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1823,7 +1823,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Limited Edition</t>
+          <t>Special Offer</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1921,7 +1921,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>New Arrival</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1971,7 +1971,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>New Arrival</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -2019,7 +2019,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Sale</t>
+          <t>Wholesale</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -2067,7 +2067,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Retail</t>
+          <t>Budget</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -2115,7 +2115,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Retail</t>
+          <t>Budget</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -2163,7 +2163,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Retail</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -2213,7 +2213,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Special Offer</t>
+          <t>Professional</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -2261,7 +2261,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Wholesale</t>
+          <t>Limited Edition</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -2311,7 +2311,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Featured</t>
+          <t>New Arrival</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -2359,7 +2359,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Special Offer</t>
+          <t>Professional</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -2409,7 +2409,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Regular</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -2457,7 +2457,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Featured</t>
+          <t>New Arrival</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -2507,7 +2507,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>Featured</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -2557,7 +2557,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Budget</t>
+          <t>On Discount</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -2605,7 +2605,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>Featured</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -2653,7 +2653,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>On Discount</t>
+          <t>Sale</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -2751,7 +2751,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>Featured</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -2801,7 +2801,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Consumer</t>
+          <t>Industrial</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -2851,7 +2851,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Professional</t>
+          <t>Clearance</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -2899,7 +2899,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Budget</t>
+          <t>On Discount</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Wholesale</t>
+          <t>Limited Edition</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -2995,7 +2995,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Limited Edition</t>
+          <t>Special Offer</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -3043,7 +3043,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Limited Edition</t>
+          <t>Special Offer</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -3091,7 +3091,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Budget</t>
+          <t>On Discount</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -3139,7 +3139,7 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Limited Edition</t>
+          <t>Special Offer</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -3189,7 +3189,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Retail</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -3239,7 +3239,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Sale  </t>
+          <t xml:space="preserve">  Wholesale  </t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -3287,7 +3287,7 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Wholesale</t>
+          <t>Limited Edition</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -3335,7 +3335,7 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Wholesale</t>
+          <t>Limited Edition</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -3383,7 +3383,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Clearance</t>
+          <t>Regular</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -3431,7 +3431,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Regular</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -3479,7 +3479,7 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Wholesale</t>
+          <t>Limited Edition</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -3527,7 +3527,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Featured</t>
+          <t>New Arrival</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -3577,7 +3577,7 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Clearance</t>
+          <t>Regular</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -3627,7 +3627,7 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Consumer</t>
+          <t>Industrial</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -3677,7 +3677,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Consumer</t>
+          <t>Industrial</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -3725,7 +3725,7 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Special Offer#</t>
+          <t>Professional#</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -3775,7 +3775,7 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Sale*</t>
+          <t>Wholesale*</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -3823,7 +3823,7 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Budget</t>
+          <t>On Discount</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -3871,7 +3871,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>Featured</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -3919,7 +3919,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Limited Edition</t>
+          <t>Special Offer</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -3969,7 +3969,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Wholesale</t>
+          <t>Limited Edition</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -4069,7 +4069,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Featured</t>
+          <t>New Arrival</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -4117,7 +4117,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Consumer</t>
+          <t>Industrial</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -4165,7 +4165,7 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Special Offer</t>
+          <t>Professional</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -4261,7 +4261,7 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Professional</t>
+          <t>Clearance</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -4309,7 +4309,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>On Discount</t>
+          <t>Sale</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -4359,7 +4359,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>On Discount</t>
+          <t>Sale</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -4407,7 +4407,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Consumer</t>
+          <t>Industrial</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -4455,7 +4455,7 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Wholesale</t>
+          <t>Limited Edition</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -4503,7 +4503,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Wholesale</t>
+          <t>Limited Edition</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -4553,7 +4553,7 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Retail</t>
+          <t>Budget</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
@@ -4601,7 +4601,7 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Professional</t>
+          <t>Clearance</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
@@ -4651,7 +4651,7 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Retail</t>
+          <t>Budget</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
@@ -4701,7 +4701,7 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Clearance</t>
+          <t>Regular</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
@@ -4749,7 +4749,7 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Budget</t>
+          <t>On Discount</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
@@ -4799,7 +4799,7 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Featured</t>
+          <t>New Arrival</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
@@ -4897,7 +4897,7 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Special Offer</t>
+          <t>Professional</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
@@ -4945,7 +4945,7 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Budget</t>
+          <t>On Discount</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
@@ -4995,7 +4995,7 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Special Offer</t>
+          <t>Professional</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
@@ -5045,7 +5045,7 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>On Discount</t>
+          <t>Sale</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
@@ -5093,7 +5093,7 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Budget</t>
+          <t>On Discount</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
@@ -5143,7 +5143,7 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Featured</t>
+          <t>New Arrival</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
@@ -5191,7 +5191,7 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Featured</t>
+          <t>New Arrival</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
@@ -5241,7 +5241,7 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Sale</t>
+          <t>Wholesale</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
@@ -5289,7 +5289,7 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Special Offer</t>
+          <t>Professional</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
@@ -5337,7 +5337,7 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Clearance</t>
+          <t>Regular</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
@@ -5366,7 +5366,7 @@
       </c>
       <c r="L101" t="inlineStr">
         <is>
-          <t>2026-01-12T19:12:03Z</t>
+          <t>2026-01-13T08:24:56Z</t>
         </is>
       </c>
     </row>
@@ -5385,7 +5385,7 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Special Offer</t>
+          <t>Professional</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
@@ -5435,7 +5435,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Clearance</t>
+          <t>Regular</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
@@ -5483,7 +5483,7 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Featured</t>
+          <t>New Arrival</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
@@ -5531,7 +5531,7 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Clearance</t>
+          <t>Regular</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
@@ -5579,7 +5579,7 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Retail</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
@@ -5629,7 +5629,7 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Regular  </t>
+          <t xml:space="preserve">  Standard  </t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
@@ -5677,7 +5677,7 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>Featured</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
@@ -5727,7 +5727,7 @@
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>Budget</t>
+          <t>On Discount</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
@@ -5775,7 +5775,7 @@
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>Budget</t>
+          <t>On Discount</t>
         </is>
       </c>
       <c r="F110" t="inlineStr">
@@ -5823,7 +5823,7 @@
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>Professional</t>
+          <t>Clearance</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
@@ -5873,7 +5873,7 @@
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Consumer</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
@@ -5921,7 +5921,7 @@
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>Limited Edition</t>
+          <t>Special Offer</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
@@ -5950,7 +5950,7 @@
       </c>
       <c r="L113" t="inlineStr">
         <is>
-          <t>2026-01-12T19:12:03Z</t>
+          <t>2026-01-13T08:24:55Z</t>
         </is>
       </c>
     </row>
@@ -5971,7 +5971,7 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>Sale</t>
+          <t>Wholesale</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
@@ -6019,7 +6019,7 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>Featured</t>
+          <t>New Arrival</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
@@ -6067,7 +6067,7 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Consumer</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
@@ -6213,7 +6213,7 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>On Discount</t>
+          <t>Sale</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
@@ -6261,7 +6261,7 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>On Discount</t>
+          <t>Sale</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
@@ -6309,7 +6309,7 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Wholesale  </t>
+          <t xml:space="preserve">  Limited Edition  </t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
@@ -6359,7 +6359,7 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>Sale</t>
+          <t>Wholesale</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
@@ -6388,7 +6388,7 @@
       </c>
       <c r="L122" t="inlineStr">
         <is>
-          <t>2026-01-12T19:12:03Z</t>
+          <t>2026-01-13T08:24:55Z</t>
         </is>
       </c>
     </row>
@@ -6407,7 +6407,7 @@
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Standard  </t>
+          <t xml:space="preserve">  Consumer  </t>
         </is>
       </c>
       <c r="F123" t="inlineStr">
@@ -6457,7 +6457,7 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>Professional</t>
+          <t>Clearance</t>
         </is>
       </c>
       <c r="F124" t="inlineStr">
@@ -6507,7 +6507,7 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>Sale</t>
+          <t>Wholesale</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
@@ -6557,7 +6557,7 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>Regular</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">
@@ -6605,7 +6605,7 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Retail</t>
         </is>
       </c>
       <c r="F127" t="inlineStr">
@@ -6653,7 +6653,7 @@
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>Limited Edition</t>
+          <t>Special Offer</t>
         </is>
       </c>
       <c r="F128" t="inlineStr">
@@ -6703,7 +6703,7 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>Featured</t>
+          <t>New Arrival</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
@@ -6753,7 +6753,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>Featured</t>
+          <t>New Arrival</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
@@ -6803,7 +6803,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Regular</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
@@ -6853,7 +6853,7 @@
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>Consumer</t>
+          <t>Industrial</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
@@ -6903,7 +6903,7 @@
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>On Discount</t>
+          <t>Sale</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
@@ -6951,7 +6951,7 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>New Arrival</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
@@ -7001,7 +7001,7 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Consumer</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
@@ -7051,7 +7051,7 @@
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>On Discount</t>
+          <t>Sale</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
@@ -7149,7 +7149,7 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Retail</t>
         </is>
       </c>
       <c r="F138" t="inlineStr">
@@ -7199,7 +7199,7 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>New Arrival</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
@@ -7247,7 +7247,7 @@
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>On Discount</t>
+          <t>Sale</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
@@ -7295,7 +7295,7 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>Sale</t>
+          <t>Wholesale</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
@@ -7343,7 +7343,7 @@
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>Special Offer</t>
+          <t>Professional</t>
         </is>
       </c>
       <c r="F142" t="inlineStr">
@@ -7391,7 +7391,7 @@
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>Budget</t>
+          <t>On Discount</t>
         </is>
       </c>
       <c r="F143" t="inlineStr">
@@ -7439,7 +7439,7 @@
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>Wholesale</t>
+          <t>Limited Edition</t>
         </is>
       </c>
       <c r="F144" t="inlineStr">
@@ -7489,7 +7489,7 @@
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>Wholesale</t>
+          <t>Limited Edition</t>
         </is>
       </c>
       <c r="F145" t="inlineStr">
@@ -7537,7 +7537,7 @@
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>Budget</t>
+          <t>On Discount</t>
         </is>
       </c>
       <c r="F146" t="inlineStr">
@@ -7566,7 +7566,7 @@
       </c>
       <c r="L146" t="inlineStr">
         <is>
-          <t>2026-01-12T19:12:03Z</t>
+          <t>2026-01-13T08:24:55Z</t>
         </is>
       </c>
     </row>
@@ -7585,7 +7585,7 @@
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>wholesale</t>
+          <t>limited edition</t>
         </is>
       </c>
       <c r="F147" t="inlineStr">
@@ -7635,7 +7635,7 @@
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>Featured</t>
         </is>
       </c>
       <c r="F148" t="inlineStr">
@@ -7685,7 +7685,7 @@
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>Clearance</t>
+          <t>Regular</t>
         </is>
       </c>
       <c r="F149" t="inlineStr">
@@ -7733,7 +7733,7 @@
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>Retail</t>
+          <t>Budget</t>
         </is>
       </c>
       <c r="F150" t="inlineStr">
@@ -7781,7 +7781,7 @@
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>On Discount</t>
+          <t>Sale</t>
         </is>
       </c>
       <c r="F151" t="inlineStr">
@@ -7831,7 +7831,7 @@
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>Budget</t>
+          <t>On Discount</t>
         </is>
       </c>
       <c r="F152" t="inlineStr">
@@ -7881,7 +7881,7 @@
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>Premium%</t>
+          <t>Featured%</t>
         </is>
       </c>
       <c r="F153" t="inlineStr">
@@ -7929,7 +7929,7 @@
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>Clearance</t>
+          <t>Regular</t>
         </is>
       </c>
       <c r="F154" t="inlineStr">
@@ -7977,7 +7977,7 @@
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>Professional</t>
+          <t>Clearance</t>
         </is>
       </c>
       <c r="F155" t="inlineStr">
@@ -8025,7 +8025,7 @@
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>On Discount</t>
+          <t>Sale</t>
         </is>
       </c>
       <c r="F156" t="inlineStr">
@@ -8075,7 +8075,7 @@
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Retail</t>
         </is>
       </c>
       <c r="F157" t="inlineStr">
@@ -8123,7 +8123,7 @@
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>Featured</t>
+          <t>New Arrival</t>
         </is>
       </c>
       <c r="F158" t="inlineStr">
@@ -8171,7 +8171,7 @@
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>Limited Edition</t>
+          <t>Special Offer</t>
         </is>
       </c>
       <c r="F159" t="inlineStr">
@@ -8219,7 +8219,7 @@
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>Limited Edition</t>
+          <t>Special Offer</t>
         </is>
       </c>
       <c r="F160" t="inlineStr">
@@ -8267,7 +8267,7 @@
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Consumer</t>
         </is>
       </c>
       <c r="F161" t="inlineStr">
@@ -8317,7 +8317,7 @@
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>Budget&amp;</t>
+          <t>On Discount&amp;</t>
         </is>
       </c>
       <c r="F162" t="inlineStr">
@@ -8365,7 +8365,7 @@
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>Professional</t>
+          <t>Clearance</t>
         </is>
       </c>
       <c r="F163" t="inlineStr">
@@ -8415,7 +8415,7 @@
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>Professional</t>
+          <t>Clearance</t>
         </is>
       </c>
       <c r="F164" t="inlineStr">
@@ -8465,7 +8465,7 @@
       </c>
       <c r="E165" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Retail  </t>
+          <t xml:space="preserve">  Budget  </t>
         </is>
       </c>
       <c r="F165" t="inlineStr">
@@ -8515,7 +8515,7 @@
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Featured  </t>
+          <t xml:space="preserve">  New Arrival  </t>
         </is>
       </c>
       <c r="F166" t="inlineStr">
@@ -8565,7 +8565,7 @@
       </c>
       <c r="E167" t="inlineStr">
         <is>
-          <t>Wholesale</t>
+          <t>Limited Edition</t>
         </is>
       </c>
       <c r="F167" t="inlineStr">
@@ -8613,7 +8613,7 @@
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>Wholesale</t>
+          <t>Limited Edition</t>
         </is>
       </c>
       <c r="F168" t="inlineStr">
@@ -8663,7 +8663,7 @@
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>Featured</t>
         </is>
       </c>
       <c r="F169" t="inlineStr">
@@ -8711,7 +8711,7 @@
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>Featured</t>
         </is>
       </c>
       <c r="F170" t="inlineStr">
@@ -8759,7 +8759,7 @@
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Consumer</t>
         </is>
       </c>
       <c r="F171" t="inlineStr">
@@ -8809,7 +8809,7 @@
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>New Arrival</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="F172" t="inlineStr">
@@ -8859,7 +8859,7 @@
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Consumer</t>
         </is>
       </c>
       <c r="F173" t="inlineStr">
@@ -8955,7 +8955,7 @@
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>Special Offer</t>
+          <t>Professional</t>
         </is>
       </c>
       <c r="F175" t="inlineStr">
@@ -9005,7 +9005,7 @@
       </c>
       <c r="E176" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Retail</t>
         </is>
       </c>
       <c r="F176" t="inlineStr">
@@ -9034,7 +9034,7 @@
       </c>
       <c r="L176" t="inlineStr">
         <is>
-          <t>2026-01-12T19:12:03Z</t>
+          <t>2026-01-13T08:24:56Z</t>
         </is>
       </c>
     </row>
@@ -9055,7 +9055,7 @@
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>Budget</t>
+          <t>On Discount</t>
         </is>
       </c>
       <c r="F177" t="inlineStr">
@@ -9105,7 +9105,7 @@
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t>Wholesale</t>
+          <t>Limited Edition</t>
         </is>
       </c>
       <c r="F178" t="inlineStr">
@@ -9153,7 +9153,7 @@
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t>Consumer</t>
+          <t>Industrial</t>
         </is>
       </c>
       <c r="F179" t="inlineStr">
@@ -9201,7 +9201,7 @@
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Retail</t>
         </is>
       </c>
       <c r="F180" t="inlineStr">
@@ -9251,7 +9251,7 @@
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Consumer</t>
         </is>
       </c>
       <c r="F181" t="inlineStr">
@@ -9299,7 +9299,7 @@
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>Regular</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="F182" t="inlineStr">
@@ -9347,7 +9347,7 @@
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>Limited Edition</t>
+          <t>Special Offer</t>
         </is>
       </c>
       <c r="F183" t="inlineStr">
@@ -9397,7 +9397,7 @@
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>Professional</t>
+          <t>Clearance</t>
         </is>
       </c>
       <c r="F184" t="inlineStr">
@@ -9447,7 +9447,7 @@
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>New Arrival</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="F185" t="inlineStr">
@@ -9495,7 +9495,7 @@
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>Special Offer</t>
+          <t>Professional</t>
         </is>
       </c>
       <c r="F186" t="inlineStr">
@@ -9543,7 +9543,7 @@
       </c>
       <c r="E187" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Retail</t>
         </is>
       </c>
       <c r="F187" t="inlineStr">
@@ -9593,7 +9593,7 @@
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>On Discount</t>
+          <t>Sale</t>
         </is>
       </c>
       <c r="F188" t="inlineStr">
@@ -9641,7 +9641,7 @@
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t>Featured</t>
+          <t>New Arrival</t>
         </is>
       </c>
       <c r="F189" t="inlineStr">
@@ -9689,7 +9689,7 @@
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>Special Offer</t>
+          <t>Professional</t>
         </is>
       </c>
       <c r="F190" t="inlineStr">
@@ -9739,7 +9739,7 @@
       </c>
       <c r="E191" t="inlineStr">
         <is>
-          <t>On Discount</t>
+          <t>Sale</t>
         </is>
       </c>
       <c r="F191" t="inlineStr">
@@ -9787,7 +9787,7 @@
       </c>
       <c r="E192" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Retail</t>
         </is>
       </c>
       <c r="F192" t="inlineStr">
@@ -9837,7 +9837,7 @@
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t>Wholesale</t>
+          <t>Limited Edition</t>
         </is>
       </c>
       <c r="F193" t="inlineStr">
@@ -9887,7 +9887,7 @@
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>PREMIUM</t>
+          <t>FEATURED</t>
         </is>
       </c>
       <c r="F194" t="inlineStr">
@@ -9937,7 +9937,7 @@
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t>Regular</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="F195" t="inlineStr">
@@ -9987,7 +9987,7 @@
       </c>
       <c r="E196" t="inlineStr">
         <is>
-          <t>On Discount</t>
+          <t>Sale</t>
         </is>
       </c>
       <c r="F196" t="inlineStr">
@@ -10035,7 +10035,7 @@
       </c>
       <c r="E197" t="inlineStr">
         <is>
-          <t>BUDGET</t>
+          <t>ON DISCOUNT</t>
         </is>
       </c>
       <c r="F197" t="inlineStr">
@@ -10085,7 +10085,7 @@
       </c>
       <c r="E198" t="inlineStr">
         <is>
-          <t>Wholesale</t>
+          <t>Limited Edition</t>
         </is>
       </c>
       <c r="F198" t="inlineStr">
@@ -10133,7 +10133,7 @@
       </c>
       <c r="E199" t="inlineStr">
         <is>
-          <t>Special Offer</t>
+          <t>Professional</t>
         </is>
       </c>
       <c r="F199" t="inlineStr">
@@ -10181,7 +10181,7 @@
       </c>
       <c r="E200" t="inlineStr">
         <is>
-          <t>Retail</t>
+          <t>Budget</t>
         </is>
       </c>
       <c r="F200" t="inlineStr">
@@ -10229,7 +10229,7 @@
       </c>
       <c r="E201" t="inlineStr">
         <is>
-          <t>On Discount</t>
+          <t>Sale</t>
         </is>
       </c>
       <c r="F201" t="inlineStr">

</xml_diff>

<commit_message>
Fixed Negative Order Profit and Massive Discounts
</commit_message>
<xml_diff>
--- a/faker/categories.xlsx
+++ b/faker/categories.xlsx
@@ -505,7 +505,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Limited Edition</t>
+          <t>Consumer</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -553,7 +553,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>On Discount</t>
+          <t>Limited Edition</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -601,7 +601,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Special Offer</t>
+          <t>Featured</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -649,7 +649,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Budget</t>
+          <t>Sale</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -697,7 +697,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>New Arrival</t>
+          <t>Clearance</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -747,7 +747,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Featured  </t>
+          <t xml:space="preserve">  Professional  </t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -797,7 +797,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Sale</t>
+          <t>New Arrival</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -847,7 +847,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Special Offer</t>
+          <t>Featured</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -895,7 +895,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>On Discount</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -945,7 +945,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Clearance</t>
+          <t>Budget</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -995,7 +995,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Regular@</t>
+          <t>Standard@</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1045,7 +1045,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>On Discount</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1093,7 +1093,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Clearance</t>
+          <t>Budget</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1141,7 +1141,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Featured</t>
+          <t>Professional</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1189,7 +1189,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1237,7 +1237,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Retail</t>
+          <t>Industrial</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1285,7 +1285,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Wholesale</t>
+          <t>Best Seller</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1335,7 +1335,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Best Seller</t>
+          <t>Regular</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1385,7 +1385,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Sale</t>
+          <t>New Arrival</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1433,7 +1433,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Special Offer</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1481,7 +1481,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Retail  </t>
+          <t xml:space="preserve">  Industrial  </t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1531,7 +1531,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>New Arrival</t>
+          <t>Clearance</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1579,7 +1579,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Professional</t>
+          <t>Wholesale</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1629,7 +1629,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Regular</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1677,7 +1677,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Retail</t>
+          <t>Industrial</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1727,7 +1727,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>INDUSTRIAL</t>
+          <t>PREMIUM</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1775,7 +1775,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Industrial  </t>
+          <t xml:space="preserve">  Premium  </t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1823,7 +1823,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Special Offer</t>
+          <t>Featured</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1871,7 +1871,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Best Seller</t>
+          <t>Regular</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1921,7 +1921,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>On Discount</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1971,7 +1971,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>On Discount</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -2019,7 +2019,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Wholesale</t>
+          <t>Best Seller</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -2067,7 +2067,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Budget</t>
+          <t>Sale</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -2115,7 +2115,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Budget</t>
+          <t>Sale</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -2163,7 +2163,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Retail</t>
+          <t>Industrial</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -2213,7 +2213,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Professional</t>
+          <t>Wholesale</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -2261,7 +2261,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Limited Edition</t>
+          <t>Consumer</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -2311,7 +2311,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>New Arrival</t>
+          <t>Clearance</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -2359,7 +2359,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Professional</t>
+          <t>Wholesale</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -2409,7 +2409,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Special Offer</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -2457,7 +2457,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>New Arrival</t>
+          <t>Clearance</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -2507,7 +2507,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Featured</t>
+          <t>Professional</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -2557,7 +2557,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>On Discount</t>
+          <t>Limited Edition</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -2605,7 +2605,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Featured</t>
+          <t>Professional</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -2653,7 +2653,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Sale</t>
+          <t>New Arrival</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -2703,7 +2703,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Best Seller</t>
+          <t>Regular</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -2751,7 +2751,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Featured</t>
+          <t>Professional</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -2801,7 +2801,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -2851,7 +2851,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Clearance</t>
+          <t>Budget</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -2899,7 +2899,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>On Discount</t>
+          <t>Limited Edition</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Limited Edition</t>
+          <t>Consumer</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -2995,7 +2995,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Special Offer</t>
+          <t>Featured</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -3043,7 +3043,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Special Offer</t>
+          <t>Featured</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -3091,7 +3091,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>On Discount</t>
+          <t>Limited Edition</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -3139,7 +3139,7 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Special Offer</t>
+          <t>Featured</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -3189,7 +3189,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Retail</t>
+          <t>Industrial</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -3239,7 +3239,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Wholesale  </t>
+          <t xml:space="preserve">  Best Seller  </t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -3287,7 +3287,7 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Limited Edition</t>
+          <t>Consumer</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -3335,7 +3335,7 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Limited Edition</t>
+          <t>Consumer</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -3383,7 +3383,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Regular</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -3431,7 +3431,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Special Offer</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -3479,7 +3479,7 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Limited Edition</t>
+          <t>Consumer</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -3527,7 +3527,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>New Arrival</t>
+          <t>Clearance</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -3577,7 +3577,7 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Regular</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -3627,7 +3627,7 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -3677,7 +3677,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -3725,7 +3725,7 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Professional#</t>
+          <t>Wholesale#</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -3775,7 +3775,7 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Wholesale*</t>
+          <t>Best Seller*</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -3823,7 +3823,7 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>On Discount</t>
+          <t>Limited Edition</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -3871,7 +3871,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Featured</t>
+          <t>Professional</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -3919,7 +3919,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Special Offer</t>
+          <t>Featured</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -3969,7 +3969,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Limited Edition</t>
+          <t>Consumer</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -4019,7 +4019,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Best Seller</t>
+          <t>Regular</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -4069,7 +4069,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>New Arrival</t>
+          <t>Clearance</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -4117,7 +4117,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -4165,7 +4165,7 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Professional</t>
+          <t>Wholesale</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -4213,7 +4213,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Best Seller</t>
+          <t>Regular</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -4261,7 +4261,7 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Clearance</t>
+          <t>Budget</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -4309,7 +4309,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Sale</t>
+          <t>New Arrival</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -4359,7 +4359,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Sale</t>
+          <t>New Arrival</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -4407,7 +4407,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -4455,7 +4455,7 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Limited Edition</t>
+          <t>Consumer</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -4503,7 +4503,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Limited Edition</t>
+          <t>Consumer</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -4553,7 +4553,7 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Budget</t>
+          <t>Sale</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
@@ -4601,7 +4601,7 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Clearance</t>
+          <t>Budget</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
@@ -4651,7 +4651,7 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Budget</t>
+          <t>Sale</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
@@ -4701,7 +4701,7 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Regular</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
@@ -4749,7 +4749,7 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>On Discount</t>
+          <t>Limited Edition</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
@@ -4799,7 +4799,7 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>New Arrival</t>
+          <t>Clearance</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
@@ -4847,7 +4847,7 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Best Seller</t>
+          <t>Regular</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
@@ -4897,7 +4897,7 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Professional</t>
+          <t>Wholesale</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
@@ -4945,7 +4945,7 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>On Discount</t>
+          <t>Limited Edition</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
@@ -4995,7 +4995,7 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Professional</t>
+          <t>Wholesale</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
@@ -5045,7 +5045,7 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Sale</t>
+          <t>New Arrival</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
@@ -5093,7 +5093,7 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>On Discount</t>
+          <t>Limited Edition</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
@@ -5143,7 +5143,7 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>New Arrival</t>
+          <t>Clearance</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
@@ -5191,7 +5191,7 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>New Arrival</t>
+          <t>Clearance</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
@@ -5241,7 +5241,7 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Wholesale</t>
+          <t>Best Seller</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
@@ -5289,7 +5289,7 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Professional</t>
+          <t>Wholesale</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
@@ -5337,7 +5337,7 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Regular</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
@@ -5366,7 +5366,7 @@
       </c>
       <c r="L101" t="inlineStr">
         <is>
-          <t>2026-01-13T08:24:56Z</t>
+          <t>2026-01-13T18:47:27Z</t>
         </is>
       </c>
     </row>
@@ -5385,7 +5385,7 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Professional</t>
+          <t>Wholesale</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
@@ -5435,7 +5435,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Regular</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
@@ -5483,7 +5483,7 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>New Arrival</t>
+          <t>Clearance</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
@@ -5531,7 +5531,7 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Regular</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
@@ -5579,7 +5579,7 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Retail</t>
+          <t>Industrial</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
@@ -5629,7 +5629,7 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Standard  </t>
+          <t xml:space="preserve">  Special Offer  </t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
@@ -5677,7 +5677,7 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Featured</t>
+          <t>Professional</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
@@ -5727,7 +5727,7 @@
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>On Discount</t>
+          <t>Limited Edition</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
@@ -5775,7 +5775,7 @@
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>On Discount</t>
+          <t>Limited Edition</t>
         </is>
       </c>
       <c r="F110" t="inlineStr">
@@ -5823,7 +5823,7 @@
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>Clearance</t>
+          <t>Budget</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
@@ -5873,7 +5873,7 @@
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>Consumer</t>
+          <t>Retail</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
@@ -5921,7 +5921,7 @@
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>Special Offer</t>
+          <t>Featured</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
@@ -5950,7 +5950,7 @@
       </c>
       <c r="L113" t="inlineStr">
         <is>
-          <t>2026-01-13T08:24:55Z</t>
+          <t>2026-01-13T18:47:27Z</t>
         </is>
       </c>
     </row>
@@ -5971,7 +5971,7 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>Wholesale</t>
+          <t>Best Seller</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
@@ -6019,7 +6019,7 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>New Arrival</t>
+          <t>Clearance</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
@@ -6067,7 +6067,7 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Consumer</t>
+          <t>Retail</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
@@ -6117,7 +6117,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Best Seller</t>
+          <t>Regular</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
@@ -6165,7 +6165,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Best Seller</t>
+          <t>Regular</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
@@ -6213,7 +6213,7 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>Sale</t>
+          <t>New Arrival</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
@@ -6261,7 +6261,7 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Sale</t>
+          <t>New Arrival</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
@@ -6309,7 +6309,7 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Limited Edition  </t>
+          <t xml:space="preserve">  Consumer  </t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
@@ -6359,7 +6359,7 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>Wholesale</t>
+          <t>Best Seller</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
@@ -6388,7 +6388,7 @@
       </c>
       <c r="L122" t="inlineStr">
         <is>
-          <t>2026-01-13T08:24:55Z</t>
+          <t>2026-01-13T18:47:27Z</t>
         </is>
       </c>
     </row>
@@ -6407,7 +6407,7 @@
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Consumer  </t>
+          <t xml:space="preserve">  Retail  </t>
         </is>
       </c>
       <c r="F123" t="inlineStr">
@@ -6457,7 +6457,7 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>Clearance</t>
+          <t>Budget</t>
         </is>
       </c>
       <c r="F124" t="inlineStr">
@@ -6507,7 +6507,7 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>Wholesale</t>
+          <t>Best Seller</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
@@ -6557,7 +6557,7 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Special Offer</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">
@@ -6605,7 +6605,7 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>Retail</t>
+          <t>Industrial</t>
         </is>
       </c>
       <c r="F127" t="inlineStr">
@@ -6653,7 +6653,7 @@
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>Special Offer</t>
+          <t>Featured</t>
         </is>
       </c>
       <c r="F128" t="inlineStr">
@@ -6703,7 +6703,7 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>New Arrival</t>
+          <t>Clearance</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
@@ -6753,7 +6753,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>New Arrival</t>
+          <t>Clearance</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
@@ -6803,7 +6803,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Special Offer</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
@@ -6853,7 +6853,7 @@
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
@@ -6903,7 +6903,7 @@
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>Sale</t>
+          <t>New Arrival</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
@@ -6951,7 +6951,7 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>On Discount</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
@@ -7001,7 +7001,7 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>Consumer</t>
+          <t>Retail</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
@@ -7051,7 +7051,7 @@
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>Sale</t>
+          <t>New Arrival</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
@@ -7099,7 +7099,7 @@
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Best Seller  </t>
+          <t xml:space="preserve">  Regular  </t>
         </is>
       </c>
       <c r="F137" t="inlineStr">
@@ -7149,7 +7149,7 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>Retail</t>
+          <t>Industrial</t>
         </is>
       </c>
       <c r="F138" t="inlineStr">
@@ -7199,7 +7199,7 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>On Discount</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
@@ -7247,7 +7247,7 @@
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>Sale</t>
+          <t>New Arrival</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
@@ -7295,7 +7295,7 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>Wholesale</t>
+          <t>Best Seller</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
@@ -7343,7 +7343,7 @@
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>Professional</t>
+          <t>Wholesale</t>
         </is>
       </c>
       <c r="F142" t="inlineStr">
@@ -7391,7 +7391,7 @@
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>On Discount</t>
+          <t>Limited Edition</t>
         </is>
       </c>
       <c r="F143" t="inlineStr">
@@ -7439,7 +7439,7 @@
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>Limited Edition</t>
+          <t>Consumer</t>
         </is>
       </c>
       <c r="F144" t="inlineStr">
@@ -7489,7 +7489,7 @@
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>Limited Edition</t>
+          <t>Consumer</t>
         </is>
       </c>
       <c r="F145" t="inlineStr">
@@ -7537,7 +7537,7 @@
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>On Discount</t>
+          <t>Limited Edition</t>
         </is>
       </c>
       <c r="F146" t="inlineStr">
@@ -7566,7 +7566,7 @@
       </c>
       <c r="L146" t="inlineStr">
         <is>
-          <t>2026-01-13T08:24:55Z</t>
+          <t>2026-01-13T18:47:27Z</t>
         </is>
       </c>
     </row>
@@ -7585,7 +7585,7 @@
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>limited edition</t>
+          <t>consumer</t>
         </is>
       </c>
       <c r="F147" t="inlineStr">
@@ -7635,7 +7635,7 @@
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>Featured</t>
+          <t>Professional</t>
         </is>
       </c>
       <c r="F148" t="inlineStr">
@@ -7685,7 +7685,7 @@
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>Regular</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="F149" t="inlineStr">
@@ -7733,7 +7733,7 @@
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>Budget</t>
+          <t>Sale</t>
         </is>
       </c>
       <c r="F150" t="inlineStr">
@@ -7781,7 +7781,7 @@
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>Sale</t>
+          <t>New Arrival</t>
         </is>
       </c>
       <c r="F151" t="inlineStr">
@@ -7831,7 +7831,7 @@
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>On Discount</t>
+          <t>Limited Edition</t>
         </is>
       </c>
       <c r="F152" t="inlineStr">
@@ -7881,7 +7881,7 @@
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>Featured%</t>
+          <t>Professional%</t>
         </is>
       </c>
       <c r="F153" t="inlineStr">
@@ -7929,7 +7929,7 @@
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>Regular</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="F154" t="inlineStr">
@@ -7977,7 +7977,7 @@
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>Clearance</t>
+          <t>Budget</t>
         </is>
       </c>
       <c r="F155" t="inlineStr">
@@ -8025,7 +8025,7 @@
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>Sale</t>
+          <t>New Arrival</t>
         </is>
       </c>
       <c r="F156" t="inlineStr">
@@ -8075,7 +8075,7 @@
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>Retail</t>
+          <t>Industrial</t>
         </is>
       </c>
       <c r="F157" t="inlineStr">
@@ -8123,7 +8123,7 @@
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>New Arrival</t>
+          <t>Clearance</t>
         </is>
       </c>
       <c r="F158" t="inlineStr">
@@ -8171,7 +8171,7 @@
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>Special Offer</t>
+          <t>Featured</t>
         </is>
       </c>
       <c r="F159" t="inlineStr">
@@ -8219,7 +8219,7 @@
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>Special Offer</t>
+          <t>Featured</t>
         </is>
       </c>
       <c r="F160" t="inlineStr">
@@ -8267,7 +8267,7 @@
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>Consumer</t>
+          <t>Retail</t>
         </is>
       </c>
       <c r="F161" t="inlineStr">
@@ -8317,7 +8317,7 @@
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>On Discount&amp;</t>
+          <t>Limited Edition&amp;</t>
         </is>
       </c>
       <c r="F162" t="inlineStr">
@@ -8365,7 +8365,7 @@
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>Clearance</t>
+          <t>Budget</t>
         </is>
       </c>
       <c r="F163" t="inlineStr">
@@ -8415,7 +8415,7 @@
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>Clearance</t>
+          <t>Budget</t>
         </is>
       </c>
       <c r="F164" t="inlineStr">
@@ -8465,7 +8465,7 @@
       </c>
       <c r="E165" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Budget  </t>
+          <t xml:space="preserve">  Sale  </t>
         </is>
       </c>
       <c r="F165" t="inlineStr">
@@ -8515,7 +8515,7 @@
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t xml:space="preserve">  New Arrival  </t>
+          <t xml:space="preserve">  Clearance  </t>
         </is>
       </c>
       <c r="F166" t="inlineStr">
@@ -8565,7 +8565,7 @@
       </c>
       <c r="E167" t="inlineStr">
         <is>
-          <t>Limited Edition</t>
+          <t>Consumer</t>
         </is>
       </c>
       <c r="F167" t="inlineStr">
@@ -8613,7 +8613,7 @@
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>Limited Edition</t>
+          <t>Consumer</t>
         </is>
       </c>
       <c r="F168" t="inlineStr">
@@ -8663,7 +8663,7 @@
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>Featured</t>
+          <t>Professional</t>
         </is>
       </c>
       <c r="F169" t="inlineStr">
@@ -8711,7 +8711,7 @@
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>Featured</t>
+          <t>Professional</t>
         </is>
       </c>
       <c r="F170" t="inlineStr">
@@ -8759,7 +8759,7 @@
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>Consumer</t>
+          <t>Retail</t>
         </is>
       </c>
       <c r="F171" t="inlineStr">
@@ -8809,7 +8809,7 @@
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>On Discount</t>
         </is>
       </c>
       <c r="F172" t="inlineStr">
@@ -8859,7 +8859,7 @@
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>Consumer</t>
+          <t>Retail</t>
         </is>
       </c>
       <c r="F173" t="inlineStr">
@@ -8907,7 +8907,7 @@
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t>Best Seller</t>
+          <t>Regular</t>
         </is>
       </c>
       <c r="F174" t="inlineStr">
@@ -8955,7 +8955,7 @@
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>Professional</t>
+          <t>Wholesale</t>
         </is>
       </c>
       <c r="F175" t="inlineStr">
@@ -9005,7 +9005,7 @@
       </c>
       <c r="E176" t="inlineStr">
         <is>
-          <t>Retail</t>
+          <t>Industrial</t>
         </is>
       </c>
       <c r="F176" t="inlineStr">
@@ -9034,7 +9034,7 @@
       </c>
       <c r="L176" t="inlineStr">
         <is>
-          <t>2026-01-13T08:24:56Z</t>
+          <t>2026-01-13T18:47:27Z</t>
         </is>
       </c>
     </row>
@@ -9055,7 +9055,7 @@
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>On Discount</t>
+          <t>Limited Edition</t>
         </is>
       </c>
       <c r="F177" t="inlineStr">
@@ -9105,7 +9105,7 @@
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t>Limited Edition</t>
+          <t>Consumer</t>
         </is>
       </c>
       <c r="F178" t="inlineStr">
@@ -9153,7 +9153,7 @@
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="F179" t="inlineStr">
@@ -9201,7 +9201,7 @@
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t>Retail</t>
+          <t>Industrial</t>
         </is>
       </c>
       <c r="F180" t="inlineStr">
@@ -9251,7 +9251,7 @@
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>Consumer</t>
+          <t>Retail</t>
         </is>
       </c>
       <c r="F181" t="inlineStr">
@@ -9299,7 +9299,7 @@
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Special Offer</t>
         </is>
       </c>
       <c r="F182" t="inlineStr">
@@ -9347,7 +9347,7 @@
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>Special Offer</t>
+          <t>Featured</t>
         </is>
       </c>
       <c r="F183" t="inlineStr">
@@ -9397,7 +9397,7 @@
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>Clearance</t>
+          <t>Budget</t>
         </is>
       </c>
       <c r="F184" t="inlineStr">
@@ -9447,7 +9447,7 @@
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>On Discount</t>
         </is>
       </c>
       <c r="F185" t="inlineStr">
@@ -9495,7 +9495,7 @@
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>Professional</t>
+          <t>Wholesale</t>
         </is>
       </c>
       <c r="F186" t="inlineStr">
@@ -9543,7 +9543,7 @@
       </c>
       <c r="E187" t="inlineStr">
         <is>
-          <t>Retail</t>
+          <t>Industrial</t>
         </is>
       </c>
       <c r="F187" t="inlineStr">
@@ -9593,7 +9593,7 @@
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>Sale</t>
+          <t>New Arrival</t>
         </is>
       </c>
       <c r="F188" t="inlineStr">
@@ -9641,7 +9641,7 @@
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t>New Arrival</t>
+          <t>Clearance</t>
         </is>
       </c>
       <c r="F189" t="inlineStr">
@@ -9689,7 +9689,7 @@
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>Professional</t>
+          <t>Wholesale</t>
         </is>
       </c>
       <c r="F190" t="inlineStr">
@@ -9739,7 +9739,7 @@
       </c>
       <c r="E191" t="inlineStr">
         <is>
-          <t>Sale</t>
+          <t>New Arrival</t>
         </is>
       </c>
       <c r="F191" t="inlineStr">
@@ -9787,7 +9787,7 @@
       </c>
       <c r="E192" t="inlineStr">
         <is>
-          <t>Retail</t>
+          <t>Industrial</t>
         </is>
       </c>
       <c r="F192" t="inlineStr">
@@ -9837,7 +9837,7 @@
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t>Limited Edition</t>
+          <t>Consumer</t>
         </is>
       </c>
       <c r="F193" t="inlineStr">
@@ -9887,7 +9887,7 @@
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>FEATURED</t>
+          <t>PROFESSIONAL</t>
         </is>
       </c>
       <c r="F194" t="inlineStr">
@@ -9937,7 +9937,7 @@
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Special Offer</t>
         </is>
       </c>
       <c r="F195" t="inlineStr">
@@ -9987,7 +9987,7 @@
       </c>
       <c r="E196" t="inlineStr">
         <is>
-          <t>Sale</t>
+          <t>New Arrival</t>
         </is>
       </c>
       <c r="F196" t="inlineStr">
@@ -10035,7 +10035,7 @@
       </c>
       <c r="E197" t="inlineStr">
         <is>
-          <t>ON DISCOUNT</t>
+          <t>LIMITED EDITION</t>
         </is>
       </c>
       <c r="F197" t="inlineStr">
@@ -10085,7 +10085,7 @@
       </c>
       <c r="E198" t="inlineStr">
         <is>
-          <t>Limited Edition</t>
+          <t>Consumer</t>
         </is>
       </c>
       <c r="F198" t="inlineStr">
@@ -10133,7 +10133,7 @@
       </c>
       <c r="E199" t="inlineStr">
         <is>
-          <t>Professional</t>
+          <t>Wholesale</t>
         </is>
       </c>
       <c r="F199" t="inlineStr">
@@ -10181,7 +10181,7 @@
       </c>
       <c r="E200" t="inlineStr">
         <is>
-          <t>Budget</t>
+          <t>Sale</t>
         </is>
       </c>
       <c r="F200" t="inlineStr">
@@ -10229,7 +10229,7 @@
       </c>
       <c r="E201" t="inlineStr">
         <is>
-          <t>Sale</t>
+          <t>New Arrival</t>
         </is>
       </c>
       <c r="F201" t="inlineStr">

</xml_diff>